<commit_message>
feat(ai): clean stage_final emotion words and purged candidates
</commit_message>
<xml_diff>
--- a/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
+++ b/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="56">
   <si>
     <t>word</t>
   </si>
@@ -46,9 +46,21 @@
     <t>calming</t>
   </si>
   <si>
+    <t>insightful</t>
+  </si>
+  <si>
     <t>breathtakingly</t>
   </si>
   <si>
+    <t>timely</t>
+  </si>
+  <si>
+    <t>choppy</t>
+  </si>
+  <si>
+    <t>inexpensive</t>
+  </si>
+  <si>
     <t>annoying</t>
   </si>
   <si>
@@ -82,9 +94,21 @@
     <t>令人平息平稳安心的</t>
   </si>
   <si>
+    <t>富有真知灼见生动的（解说评价）</t>
+  </si>
+  <si>
     <t>令人屏息震撼地</t>
   </si>
   <si>
+    <t>及时周到高效的</t>
+  </si>
+  <si>
+    <t>颠簸起伏不平的（颠簸体验评价）</t>
+  </si>
+  <si>
+    <t>经济实惠划算的</t>
+  </si>
+  <si>
     <t>令人烦躁恼火的</t>
   </si>
   <si>
@@ -124,7 +148,22 @@
     <t>review_348b4aff02fdf2a7c1edf068 :: We had a once in a lifetime experience on Westwind's Signature Grand Canyon South and Ground Tour. I have a terrible fear of flying but I was desperate to be able to do this tour. ...</t>
   </si>
   <si>
+    <t>review_5bd36d2b98638d7b4db8f759 :: Wow! Is what comes to mind when thinking about the experience we had with Grand Canyon Landmarks Tour by Airplane. Despite a very windy day, our pilot decided it was safe enough to...</t>
+  </si>
+  <si>
     <t>review_f2ca54d8c40cde99c66061bf :: it was an amazing experience. Staff was really nice and welcoming. Pilot was really experienced, he warned us before every bumps, it was really smooth. On the other side, the tour ...</t>
+  </si>
+  <si>
+    <t>review_6547e92113e25bfa449a9d82 :: All communication with West Winds was clear and timely.  Wyatt and Rob, our pilots were top notch, fun, informative and friendly.  We highly recommend this company!...</t>
+  </si>
+  <si>
+    <t>review_2fa849492d02f429fc735d07 :: Amazing. Very choppy with turbulence but worth every penny to see that awe inspiring view from above. 
+A memory for me to cherish as both my grown up sons with me...</t>
+  </si>
+  <si>
+    <t>review_28efb948a887db7190d66ddb :: Trip Reserved: Grand Canyon Deluxe with Hummer
+Our Group: 2 families (4 adults, 2 teenage boys)
+On a recent trip to Las Vegas, we wanted the views of the South Rim without the 9 h...</t>
   </si>
   <si>
     <t>review_18e608403c49b24b1b1be5a7 :: Since posting my original review a few weeks ago, Maui Plane Rides reached out to see if there was anything they could do to improve my 3-star experience. I appreciate the follow-u...</t>
@@ -503,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -531,10 +570,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D2">
         <v>339</v>
@@ -543,7 +582,7 @@
         <v>328</v>
       </c>
       <c r="F2" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -551,10 +590,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D3">
         <v>185</v>
@@ -563,7 +602,7 @@
         <v>182</v>
       </c>
       <c r="F3" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -571,10 +610,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D4">
         <v>138</v>
@@ -583,7 +622,7 @@
         <v>138</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -591,10 +630,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D5">
         <v>42</v>
@@ -603,7 +642,7 @@
         <v>39</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -611,10 +650,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D6">
         <v>28</v>
@@ -623,7 +662,7 @@
         <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -631,19 +670,19 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D7">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="E7">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -651,19 +690,19 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D8">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E8">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -671,19 +710,19 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D9">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="E9">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -691,19 +730,19 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D10">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="E10">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="F10" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -711,19 +750,19 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D11">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E11">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -731,19 +770,19 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D12">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F12" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -751,19 +790,99 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14">
+        <v>7</v>
+      </c>
+      <c r="E14">
+        <v>7</v>
+      </c>
+      <c r="F14" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15">
+        <v>6</v>
+      </c>
+      <c r="E15">
+        <v>6</v>
+      </c>
+      <c r="F15" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <v>5</v>
+      </c>
+      <c r="F16" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17">
         <v>4</v>
       </c>
-      <c r="E13">
+      <c r="E17">
         <v>4</v>
       </c>
-      <c r="F13" t="s">
-        <v>43</v>
+      <c r="F17" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): purge timely from clean emotion lexicons and update json config
</commit_message>
<xml_diff>
--- a/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
+++ b/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="53">
   <si>
     <t>word</t>
   </si>
@@ -52,9 +52,6 @@
     <t>breathtakingly</t>
   </si>
   <si>
-    <t>timely</t>
-  </si>
-  <si>
     <t>choppy</t>
   </si>
   <si>
@@ -100,9 +97,6 @@
     <t>令人屏息震撼地</t>
   </si>
   <si>
-    <t>及时周到高效的</t>
-  </si>
-  <si>
     <t>颠簸起伏不平的（颠簸体验评价）</t>
   </si>
   <si>
@@ -152,9 +146,6 @@
   </si>
   <si>
     <t>review_f2ca54d8c40cde99c66061bf :: it was an amazing experience. Staff was really nice and welcoming. Pilot was really experienced, he warned us before every bumps, it was really smooth. On the other side, the tour ...</t>
-  </si>
-  <si>
-    <t>review_6547e92113e25bfa449a9d82 :: All communication with West Winds was clear and timely.  Wyatt and Rob, our pilots were top notch, fun, informative and friendly.  We highly recommend this company!...</t>
   </si>
   <si>
     <t>review_2fa849492d02f429fc735d07 :: Amazing. Very choppy with turbulence but worth every penny to see that awe inspiring view from above. 
@@ -542,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -570,10 +561,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D2">
         <v>339</v>
@@ -582,7 +573,7 @@
         <v>328</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -590,10 +581,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D3">
         <v>185</v>
@@ -602,7 +593,7 @@
         <v>182</v>
       </c>
       <c r="F3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -610,10 +601,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D4">
         <v>138</v>
@@ -622,7 +613,7 @@
         <v>138</v>
       </c>
       <c r="F4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -630,10 +621,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D5">
         <v>42</v>
@@ -642,7 +633,7 @@
         <v>39</v>
       </c>
       <c r="F5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -650,10 +641,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D6">
         <v>28</v>
@@ -662,7 +653,7 @@
         <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -670,10 +661,10 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D7">
         <v>28</v>
@@ -682,7 +673,7 @@
         <v>28</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -690,19 +681,19 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D8">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E8">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -710,10 +701,10 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D9">
         <v>23</v>
@@ -722,7 +713,7 @@
         <v>22</v>
       </c>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -730,19 +721,19 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D10">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E10">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -750,19 +741,19 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -770,19 +761,19 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D12">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E12">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -790,19 +781,19 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -810,19 +801,19 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -830,19 +821,19 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -850,39 +841,19 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" t="s">
-        <v>39</v>
-      </c>
-      <c r="D17">
-        <v>4</v>
-      </c>
-      <c r="E17">
-        <v>4</v>
-      </c>
-      <c r="F17" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): apply strict human adjudication rules for stage_final emotion lexicon
</commit_message>
<xml_diff>
--- a/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
+++ b/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>word</t>
   </si>
@@ -34,42 +34,15 @@
     <t>example_context</t>
   </si>
   <si>
-    <t>beyond</t>
-  </si>
-  <si>
-    <t>mahalo</t>
-  </si>
-  <si>
-    <t>heartbeat</t>
-  </si>
-  <si>
     <t>calming</t>
   </si>
   <si>
-    <t>insightful</t>
-  </si>
-  <si>
     <t>breathtakingly</t>
   </si>
   <si>
-    <t>choppy</t>
-  </si>
-  <si>
-    <t>inexpensive</t>
-  </si>
-  <si>
     <t>annoying</t>
   </si>
   <si>
-    <t>overpriced</t>
-  </si>
-  <si>
-    <t>seamlessly</t>
-  </si>
-  <si>
-    <t>invaluable</t>
-  </si>
-  <si>
     <t>sublime</t>
   </si>
   <si>
@@ -79,94 +52,37 @@
     <t>tranquil</t>
   </si>
   <si>
-    <t>超越预期的（beyond expectations/nice）</t>
-  </si>
-  <si>
-    <t>夏威夷热忱感激之意</t>
-  </si>
-  <si>
-    <t>毫不犹豫极赞体验的（in a heartbeat）</t>
-  </si>
-  <si>
-    <t>令人平息平稳安心的</t>
-  </si>
-  <si>
-    <t>富有真知灼见生动的（解说评价）</t>
-  </si>
-  <si>
-    <t>令人屏息震撼地</t>
-  </si>
-  <si>
-    <t>颠簸起伏不平的（颠簸体验评价）</t>
-  </si>
-  <si>
-    <t>经济实惠划算的</t>
-  </si>
-  <si>
-    <t>令人烦躁恼火的</t>
-  </si>
-  <si>
-    <t>价格偏高离谱的</t>
-  </si>
-  <si>
-    <t>无缝顺畅地</t>
-  </si>
-  <si>
-    <t>弥足珍贵的</t>
-  </si>
-  <si>
-    <t>崇高壮丽绝美的</t>
-  </si>
-  <si>
-    <t>令人压力重重焦虑的</t>
-  </si>
-  <si>
-    <t>清幽宁静的</t>
+    <t>令人平息平稳安心的（Calmness State）</t>
+  </si>
+  <si>
+    <t>令人屏息震撼地（Awe/Amazement Emotion）</t>
+  </si>
+  <si>
+    <t>令人烦躁恼火的（Annoyance/Irritation Emotion）</t>
+  </si>
+  <si>
+    <t>崇高壮丽绝美的（Aesthetic Emotion/Awe）</t>
+  </si>
+  <si>
+    <t>令人压力重重焦虑的（Stress/Anxiety State）</t>
+  </si>
+  <si>
+    <t>清幽宁静的（Calmness/Serenity State）</t>
+  </si>
+  <si>
+    <t>E1_State (Direct Internal Affective State)</t>
   </si>
   <si>
     <t>E2_Appraisal (Stimulus/Service Attribute)</t>
   </si>
   <si>
-    <t>E1_State (Direct Internal Affective State)</t>
-  </si>
-  <si>
-    <t>review_72e4871b346c17114821b344 :: Was an amazing experience. Everyone we dealt with was beyond nice and helpful. Our pilot, Noah, was wonderful and helped ease our nervous children. The overhead views were spectacu...</t>
-  </si>
-  <si>
-    <t>review_612b62647c7a9935a93fdef3 :: We had an absolute amazing time. Our pilot Eric was the best!  Will be back again to see more of Maui!  Thank you for the wonderful memories. Mahalo!...</t>
-  </si>
-  <si>
-    <t>review_b562aa1c118a8a327cc24d3b :: This was by far one of the best tours I have ever been on. The experience was great from start to finish. Westwind was great to work with and Brandon took excellent care of us in t...</t>
-  </si>
-  <si>
     <t>review_348b4aff02fdf2a7c1edf068 :: We had a once in a lifetime experience on Westwind's Signature Grand Canyon South and Ground Tour. I have a terrible fear of flying but I was desperate to be able to do this tour. ...</t>
   </si>
   <si>
-    <t>review_5bd36d2b98638d7b4db8f759 :: Wow! Is what comes to mind when thinking about the experience we had with Grand Canyon Landmarks Tour by Airplane. Despite a very windy day, our pilot decided it was safe enough to...</t>
-  </si>
-  <si>
     <t>review_f2ca54d8c40cde99c66061bf :: it was an amazing experience. Staff was really nice and welcoming. Pilot was really experienced, he warned us before every bumps, it was really smooth. On the other side, the tour ...</t>
   </si>
   <si>
-    <t>review_2fa849492d02f429fc735d07 :: Amazing. Very choppy with turbulence but worth every penny to see that awe inspiring view from above. 
-A memory for me to cherish as both my grown up sons with me...</t>
-  </si>
-  <si>
-    <t>review_28efb948a887db7190d66ddb :: Trip Reserved: Grand Canyon Deluxe with Hummer
-Our Group: 2 families (4 adults, 2 teenage boys)
-On a recent trip to Las Vegas, we wanted the views of the South Rim without the 9 h...</t>
-  </si>
-  <si>
     <t>review_18e608403c49b24b1b1be5a7 :: Since posting my original review a few weeks ago, Maui Plane Rides reached out to see if there was anything they could do to improve my 3-star experience. I appreciate the follow-u...</t>
-  </si>
-  <si>
-    <t>review_6ddfeb26690a6278386a224a :: Short version: amateur, unprofessional, overpriced, uncomfortable, rude, terrible experience. Spend the extra money and take a he'll ride, or at least use a different plane ride pr...</t>
-  </si>
-  <si>
-    <t>review_dc07ab5af7d3221f30156578 :: We loved everything about this! The seaplane company coordinated seamlessly with the whale watching tour company. It was easy to get to the Renton airport via Uber from downtown Se...</t>
-  </si>
-  <si>
-    <t>review_9a14597b73a4bf02195ef793 :: We booked the Denali Flyer tour without a glacier landing, and is was a once in a lifetime experience!  We originally had the tour booked for 8/25/17, but when we arrived at K2 fro...</t>
   </si>
   <si>
     <t>review_9d1f6ad84d606ddca5e4e615 :: This flight was great and the narration was really very interesting and the landing was just sublime...</t>
@@ -533,7 +449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -561,19 +477,19 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="D2">
-        <v>339</v>
+        <v>42</v>
       </c>
       <c r="E2">
-        <v>328</v>
+        <v>39</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -581,19 +497,19 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="D3">
-        <v>185</v>
+        <v>28</v>
       </c>
       <c r="E3">
-        <v>182</v>
+        <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -601,19 +517,19 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="D4">
-        <v>138</v>
+        <v>15</v>
       </c>
       <c r="E4">
-        <v>138</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -621,19 +537,19 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="D5">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="E5">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F5" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -641,19 +557,19 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="D6">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -661,199 +577,19 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="D7">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="E7">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8">
-        <v>23</v>
-      </c>
-      <c r="E8">
-        <v>22</v>
-      </c>
-      <c r="F8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9">
-        <v>23</v>
-      </c>
-      <c r="E9">
-        <v>22</v>
-      </c>
-      <c r="F9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10">
-        <v>15</v>
-      </c>
-      <c r="E10">
-        <v>15</v>
-      </c>
-      <c r="F10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11">
-        <v>14</v>
-      </c>
-      <c r="E11">
-        <v>14</v>
-      </c>
-      <c r="F11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12">
-        <v>8</v>
-      </c>
-      <c r="E12">
-        <v>8</v>
-      </c>
-      <c r="F12" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13">
-        <v>7</v>
-      </c>
-      <c r="E13">
-        <v>7</v>
-      </c>
-      <c r="F13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14">
-        <v>6</v>
-      </c>
-      <c r="E14">
-        <v>6</v>
-      </c>
-      <c r="F14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15">
-        <v>5</v>
-      </c>
-      <c r="E15">
-        <v>5</v>
-      </c>
-      <c r="F15" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" t="s">
-        <v>37</v>
-      </c>
-      <c r="D16">
-        <v>4</v>
-      </c>
-      <c r="E16">
-        <v>4</v>
-      </c>
-      <c r="F16" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): add captivating, daunting, harrowing to emotion lexicon codebooks
</commit_message>
<xml_diff>
--- a/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
+++ b/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="254">
   <si>
     <t>word</t>
   </si>
@@ -61,21 +61,21 @@
     <t>stunned</t>
   </si>
   <si>
+    <t>cherished</t>
+  </si>
+  <si>
+    <t>mesmerized</t>
+  </si>
+  <si>
+    <t>dissapointed</t>
+  </si>
+  <si>
+    <t>frightened</t>
+  </si>
+  <si>
     <t>shocked</t>
   </si>
   <si>
-    <t>dissapointed</t>
-  </si>
-  <si>
-    <t>frightened</t>
-  </si>
-  <si>
-    <t>cherished</t>
-  </si>
-  <si>
-    <t>mesmerized</t>
-  </si>
-  <si>
     <t>claustrophobia</t>
   </si>
   <si>
@@ -85,162 +85,171 @@
     <t>panic</t>
   </si>
   <si>
+    <t>fascinated</t>
+  </si>
+  <si>
+    <t>relief</t>
+  </si>
+  <si>
+    <t>timid</t>
+  </si>
+  <si>
+    <t>amaze</t>
+  </si>
+  <si>
     <t>sublime</t>
   </si>
   <si>
-    <t>amaze</t>
-  </si>
-  <si>
-    <t>fascinated</t>
-  </si>
-  <si>
-    <t>relief</t>
-  </si>
-  <si>
-    <t>timid</t>
+    <t>marveled</t>
+  </si>
+  <si>
+    <t>stressful</t>
+  </si>
+  <si>
+    <t>hates</t>
+  </si>
+  <si>
+    <t>shock</t>
+  </si>
+  <si>
+    <t>exhilerating</t>
+  </si>
+  <si>
+    <t>apprehension</t>
+  </si>
+  <si>
+    <t>hated</t>
+  </si>
+  <si>
+    <t>envy</t>
+  </si>
+  <si>
+    <t>pity</t>
+  </si>
+  <si>
+    <t>jitters</t>
+  </si>
+  <si>
+    <t>comforted</t>
   </si>
   <si>
     <t>wowed</t>
   </si>
   <si>
-    <t>comforted</t>
-  </si>
-  <si>
-    <t>jitters</t>
-  </si>
-  <si>
-    <t>pity</t>
-  </si>
-  <si>
-    <t>envy</t>
-  </si>
-  <si>
-    <t>hated</t>
-  </si>
-  <si>
-    <t>marveled</t>
-  </si>
-  <si>
-    <t>exhilerating</t>
-  </si>
-  <si>
-    <t>apprehension</t>
-  </si>
-  <si>
-    <t>shock</t>
-  </si>
-  <si>
-    <t>hates</t>
-  </si>
-  <si>
-    <t>stressful</t>
+    <t>phobia</t>
+  </si>
+  <si>
+    <t>captivating</t>
+  </si>
+  <si>
+    <t>tranquil</t>
+  </si>
+  <si>
+    <t>peacefulness</t>
+  </si>
+  <si>
+    <t>stoked</t>
+  </si>
+  <si>
+    <t>irritating</t>
   </si>
   <si>
     <t>regretting</t>
   </si>
   <si>
+    <t>spellbound</t>
+  </si>
+  <si>
+    <t>suprised</t>
+  </si>
+  <si>
+    <t>exhilarated</t>
+  </si>
+  <si>
+    <t>underwhelmed</t>
+  </si>
+  <si>
     <t>giddy</t>
   </si>
   <si>
-    <t>underwhelmed</t>
-  </si>
-  <si>
-    <t>exhilarated</t>
-  </si>
-  <si>
-    <t>suprised</t>
-  </si>
-  <si>
     <t>dreaded</t>
   </si>
   <si>
-    <t>spellbound</t>
-  </si>
-  <si>
-    <t>phobia</t>
-  </si>
-  <si>
-    <t>irritating</t>
-  </si>
-  <si>
-    <t>stoked</t>
-  </si>
-  <si>
-    <t>peacefulness</t>
-  </si>
-  <si>
-    <t>tranquil</t>
+    <t>aprehensive</t>
+  </si>
+  <si>
+    <t>daunting</t>
+  </si>
+  <si>
+    <t>sympathy</t>
+  </si>
+  <si>
+    <t>sickening</t>
+  </si>
+  <si>
+    <t>guilty</t>
+  </si>
+  <si>
+    <t>compassionate</t>
+  </si>
+  <si>
+    <t>yay</t>
+  </si>
+  <si>
+    <t>compassion</t>
+  </si>
+  <si>
+    <t>overjoyed</t>
+  </si>
+  <si>
+    <t>remorse</t>
+  </si>
+  <si>
+    <t>suprise</t>
+  </si>
+  <si>
+    <t>ecstasy</t>
+  </si>
+  <si>
+    <t>apprehensions</t>
+  </si>
+  <si>
+    <t>astounded</t>
+  </si>
+  <si>
+    <t>ambivalent</t>
+  </si>
+  <si>
+    <t>astonished</t>
+  </si>
+  <si>
+    <t>unsettled</t>
+  </si>
+  <si>
+    <t>uneasiness</t>
   </si>
   <si>
     <t>dazzled</t>
   </si>
   <si>
-    <t>uneasiness</t>
-  </si>
-  <si>
-    <t>unsettled</t>
-  </si>
-  <si>
-    <t>astonished</t>
-  </si>
-  <si>
-    <t>ambivalent</t>
-  </si>
-  <si>
-    <t>astounded</t>
-  </si>
-  <si>
-    <t>apprehensions</t>
-  </si>
-  <si>
-    <t>ecstasy</t>
-  </si>
-  <si>
-    <t>remorse</t>
-  </si>
-  <si>
-    <t>suprise</t>
-  </si>
-  <si>
-    <t>aprehensive</t>
-  </si>
-  <si>
-    <t>overjoyed</t>
-  </si>
-  <si>
-    <t>compassion</t>
-  </si>
-  <si>
-    <t>yay</t>
-  </si>
-  <si>
-    <t>compassionate</t>
-  </si>
-  <si>
-    <t>guilty</t>
-  </si>
-  <si>
-    <t>sickening</t>
-  </si>
-  <si>
-    <t>sympathy</t>
+    <t>harrowing</t>
   </si>
   <si>
     <t>worry</t>
   </si>
   <si>
+    <t>cherish</t>
+  </si>
+  <si>
     <t>disappointed</t>
   </si>
   <si>
-    <t>cherish</t>
+    <t>marvel</t>
   </si>
   <si>
     <t>hate</t>
   </si>
   <si>
-    <t>marvel</t>
-  </si>
-  <si>
     <t>exhilarating</t>
   </si>
   <si>
@@ -253,12 +262,12 @@
     <t>dread</t>
   </si>
   <si>
+    <t>apprehensive</t>
+  </si>
+  <si>
     <t>surprise</t>
   </si>
   <si>
-    <t>apprehensive</t>
-  </si>
-  <si>
     <t>令人平息平稳安心的（Calmness State）</t>
   </si>
   <si>
@@ -280,21 +289,21 @@
     <t>感到目瞪口呆震撼的</t>
   </si>
   <si>
+    <t>珍视铭记的</t>
+  </si>
+  <si>
+    <t>被深深吸引迷住的</t>
+  </si>
+  <si>
+    <t>感到失望的（错别字变体）</t>
+  </si>
+  <si>
+    <t>感到受惊吓害怕的</t>
+  </si>
+  <si>
     <t>感到震惊惊吓的</t>
   </si>
   <si>
-    <t>感到失望的（错别字变体）</t>
-  </si>
-  <si>
-    <t>感到受惊吓害怕的</t>
-  </si>
-  <si>
-    <t>珍视铭记的</t>
-  </si>
-  <si>
-    <t>被深深吸引迷住的</t>
-  </si>
-  <si>
     <t>幽闭恐惧症（密闭机舱焦虑）</t>
   </si>
   <si>
@@ -304,145 +313,154 @@
     <t>恐慌 / 惊恐状态</t>
   </si>
   <si>
+    <t>深深入迷为之倾倒的</t>
+  </si>
+  <si>
+    <t>轻松如释重负感</t>
+  </si>
+  <si>
+    <t>胆怯害羞的</t>
+  </si>
+  <si>
+    <t>使惊叹 / 惊奇</t>
+  </si>
+  <si>
     <t>崇高壮丽绝美的（Aesthetic Emotion/Awe）</t>
   </si>
   <si>
-    <t>使惊叹 / 惊奇</t>
-  </si>
-  <si>
-    <t>深深入迷为之倾倒的</t>
-  </si>
-  <si>
-    <t>轻松如释重负感</t>
-  </si>
-  <si>
-    <t>胆怯害羞的</t>
+    <t>惊叹赞赏的</t>
+  </si>
+  <si>
+    <t>令人压力重重焦虑的（Stress/Anxiety State）</t>
+  </si>
+  <si>
+    <t>厌恶 / 讨厌</t>
+  </si>
+  <si>
+    <t>震惊 / 冲击</t>
+  </si>
+  <si>
+    <t>令人兴奋刺激酣畅地（错别字变体）</t>
+  </si>
+  <si>
+    <t>忧虑 / 疑虑不安</t>
+  </si>
+  <si>
+    <t>讨厌 / 极为憎恶的</t>
+  </si>
+  <si>
+    <t>羡慕 / 嫉妒</t>
+  </si>
+  <si>
+    <t>遗憾 / 同情怜悯</t>
+  </si>
+  <si>
+    <t>忐忑不安 / 紧张发抖感</t>
+  </si>
+  <si>
+    <t>感到安慰安心的</t>
   </si>
   <si>
     <t>被深深惊叹震撼的</t>
   </si>
   <si>
-    <t>感到安慰安心的</t>
-  </si>
-  <si>
-    <t>忐忑不安 / 紧张发抖感</t>
-  </si>
-  <si>
-    <t>遗憾 / 同情怜悯</t>
-  </si>
-  <si>
-    <t>羡慕 / 嫉妒</t>
-  </si>
-  <si>
-    <t>讨厌 / 极为憎恶的</t>
-  </si>
-  <si>
-    <t>惊叹赞赏的</t>
-  </si>
-  <si>
-    <t>令人兴奋刺激酣畅地（错别字变体）</t>
-  </si>
-  <si>
-    <t>忧虑 / 疑虑不安</t>
-  </si>
-  <si>
-    <t>震惊 / 冲击</t>
-  </si>
-  <si>
-    <t>厌恶 / 讨厌</t>
-  </si>
-  <si>
-    <t>令人压力重重焦虑的（Stress/Anxiety State）</t>
+    <t>恐惧症 / 恐高心理</t>
+  </si>
+  <si>
+    <t>扣人心弦引人入胜的</t>
+  </si>
+  <si>
+    <t>清幽宁静的（Calmness/Serenity State）</t>
+  </si>
+  <si>
+    <t>宁静详和感</t>
+  </si>
+  <si>
+    <t>极为激动期待的</t>
+  </si>
+  <si>
+    <t>令人烦躁恼火的</t>
   </si>
   <si>
     <t>感到后悔遗憾的</t>
   </si>
   <si>
+    <t>出神为之入迷的</t>
+  </si>
+  <si>
+    <t>感到惊喜惊讶的（错别字变体）</t>
+  </si>
+  <si>
+    <t>感到无比兴奋酣畅的</t>
+  </si>
+  <si>
+    <t>大失所望未达预期的</t>
+  </si>
+  <si>
     <t>兴奋得头晕目眩欢欣的</t>
   </si>
   <si>
-    <t>大失所望未达预期的</t>
-  </si>
-  <si>
-    <t>感到无比兴奋酣畅的</t>
-  </si>
-  <si>
-    <t>感到惊喜惊讶的（错别字变体）</t>
-  </si>
-  <si>
     <t>令人害怕恐惧的 / 提心吊胆</t>
   </si>
   <si>
-    <t>出神为之入迷的</t>
-  </si>
-  <si>
-    <t>恐惧症 / 恐高心理</t>
-  </si>
-  <si>
-    <t>令人烦躁恼火的</t>
-  </si>
-  <si>
-    <t>极为激动期待的</t>
-  </si>
-  <si>
-    <t>宁静详和感</t>
-  </si>
-  <si>
-    <t>清幽宁静的（Calmness/Serenity State）</t>
+    <t>感到忧虑不安的（错别字变体）</t>
+  </si>
+  <si>
+    <t>令人望而生畏胆怯的</t>
+  </si>
+  <si>
+    <t>同情 / 体谅</t>
+  </si>
+  <si>
+    <t>令人作呕恶心的</t>
+  </si>
+  <si>
+    <t>内疚内疚感</t>
+  </si>
+  <si>
+    <t>富有同理心体贴的</t>
+  </si>
+  <si>
+    <t>欢呼太棒了（情绪感叹）</t>
+  </si>
+  <si>
+    <t>同理心 / 关切</t>
+  </si>
+  <si>
+    <t>欣喜若狂的</t>
+  </si>
+  <si>
+    <t>懊悔 / 悔恨</t>
+  </si>
+  <si>
+    <t>惊喜 / 意料之外（错别字变体）</t>
+  </si>
+  <si>
+    <t>狂喜 / 极乐状态</t>
+  </si>
+  <si>
+    <t>顾虑 / 忧虑不安</t>
+  </si>
+  <si>
+    <t>感到十分震惊震撼的</t>
+  </si>
+  <si>
+    <t>矛盾复杂心理的</t>
+  </si>
+  <si>
+    <t>感到十分惊异惊叹的</t>
+  </si>
+  <si>
+    <t>心神不宁忐忑的</t>
+  </si>
+  <si>
+    <t>不安 / 忐忑感</t>
   </si>
   <si>
     <t>目眩神迷震撼的</t>
   </si>
   <si>
-    <t>不安 / 忐忑感</t>
-  </si>
-  <si>
-    <t>心神不宁忐忑的</t>
-  </si>
-  <si>
-    <t>感到十分惊异惊叹的</t>
-  </si>
-  <si>
-    <t>矛盾复杂心理的</t>
-  </si>
-  <si>
-    <t>感到十分震惊震撼的</t>
-  </si>
-  <si>
-    <t>顾虑 / 忧虑不安</t>
-  </si>
-  <si>
-    <t>狂喜 / 极乐状态</t>
-  </si>
-  <si>
-    <t>懊悔 / 悔恨</t>
-  </si>
-  <si>
-    <t>惊喜 / 意料之外（错别字变体）</t>
-  </si>
-  <si>
-    <t>感到忧虑不安的（错别字变体）</t>
-  </si>
-  <si>
-    <t>欣喜若狂的</t>
-  </si>
-  <si>
-    <t>同理心 / 关切</t>
-  </si>
-  <si>
-    <t>欢呼太棒了（情绪感叹）</t>
-  </si>
-  <si>
-    <t>富有同理心体贴的</t>
-  </si>
-  <si>
-    <t>内疚内疚感</t>
-  </si>
-  <si>
-    <t>令人作呕恶心的</t>
-  </si>
-  <si>
-    <t>同情 / 体谅</t>
+    <t>令人触目惊心惊恐的</t>
   </si>
   <si>
     <t>Unclassified</t>
@@ -460,114 +478,114 @@
     <t>Surprise / Amazement</t>
   </si>
   <si>
+    <t>Fascination / Awe</t>
+  </si>
+  <si>
+    <t>Disappointment</t>
+  </si>
+  <si>
+    <t>Fear</t>
+  </si>
+  <si>
     <t>Surprise / Shock</t>
   </si>
   <si>
-    <t>Disappointment</t>
-  </si>
-  <si>
-    <t>Fear</t>
-  </si>
-  <si>
-    <t>Fascination / Awe</t>
-  </si>
-  <si>
     <t>Fear / Anxiety</t>
   </si>
   <si>
     <t>Fear / Panic</t>
   </si>
   <si>
+    <t>Fascination</t>
+  </si>
+  <si>
+    <t>Relief</t>
+  </si>
+  <si>
+    <t>Fear / Nervousness</t>
+  </si>
+  <si>
     <t>Amazement</t>
   </si>
   <si>
-    <t>Fascination</t>
-  </si>
-  <si>
-    <t>Relief</t>
-  </si>
-  <si>
-    <t>Fear / Nervousness</t>
+    <t>Wonder / Awe</t>
+  </si>
+  <si>
+    <t>Anger / Dislike</t>
+  </si>
+  <si>
+    <t>Excitement</t>
+  </si>
+  <si>
+    <t>Anxiety / Fear</t>
+  </si>
+  <si>
+    <t>Envy</t>
+  </si>
+  <si>
+    <t>Pity / Sadness</t>
+  </si>
+  <si>
+    <t>Nervousness / Anxiety</t>
+  </si>
+  <si>
+    <t>Comfort / Relief</t>
   </si>
   <si>
     <t>Amazement / Awe</t>
   </si>
   <si>
-    <t>Comfort / Relief</t>
-  </si>
-  <si>
-    <t>Nervousness / Anxiety</t>
-  </si>
-  <si>
-    <t>Pity / Sadness</t>
-  </si>
-  <si>
-    <t>Envy</t>
-  </si>
-  <si>
-    <t>Anger / Dislike</t>
-  </si>
-  <si>
-    <t>Wonder / Awe</t>
-  </si>
-  <si>
-    <t>Excitement</t>
-  </si>
-  <si>
-    <t>Anxiety / Fear</t>
+    <t>Calm / Serenity</t>
+  </si>
+  <si>
+    <t>Annoyance / Irritation</t>
   </si>
   <si>
     <t>Regret</t>
   </si>
   <si>
+    <t>Surprise</t>
+  </si>
+  <si>
     <t>Excitement / Joy</t>
   </si>
   <si>
-    <t>Surprise</t>
-  </si>
-  <si>
     <t>Fear / Dread</t>
   </si>
   <si>
-    <t>Annoyance / Irritation</t>
-  </si>
-  <si>
-    <t>Calm / Serenity</t>
+    <t>Sympathy</t>
+  </si>
+  <si>
+    <t>Disgust</t>
+  </si>
+  <si>
+    <t>Guilt</t>
+  </si>
+  <si>
+    <t>Compassion</t>
+  </si>
+  <si>
+    <t>Joy / Excitement</t>
+  </si>
+  <si>
+    <t>Regret / Guilt</t>
+  </si>
+  <si>
+    <t>Intense Joy</t>
+  </si>
+  <si>
+    <t>Mixed Emotion</t>
+  </si>
+  <si>
+    <t>Amazement / Surprise</t>
+  </si>
+  <si>
+    <t>Uneasiness / Anxiety</t>
   </si>
   <si>
     <t>Anxiety</t>
   </si>
   <si>
-    <t>Uneasiness / Anxiety</t>
-  </si>
-  <si>
-    <t>Amazement / Surprise</t>
-  </si>
-  <si>
-    <t>Mixed Emotion</t>
-  </si>
-  <si>
-    <t>Intense Joy</t>
-  </si>
-  <si>
-    <t>Regret / Guilt</t>
-  </si>
-  <si>
-    <t>Compassion</t>
-  </si>
-  <si>
-    <t>Joy / Excitement</t>
-  </si>
-  <si>
-    <t>Guilt</t>
-  </si>
-  <si>
-    <t>Disgust</t>
-  </si>
-  <si>
-    <t>Sympathy</t>
-  </si>
-  <si>
     <t>E1_State (Direct Internal Affective State)</t>
   </si>
   <si>
@@ -593,24 +611,24 @@
   </si>
   <si>
     <t>review_abb78201714fed1e189fb212 :: After several days of rain, we were driving into Talkeetna to take the Hurricane Turn train, but as we topped the hill leading down into town, we were stunned to see clear skies ov...</t>
+  </si>
+  <si>
+    <t>review_b1f4591ba3fe0c7697725cd4 :: Just an incredible time and an experience to be cherished. We had a lot of fun and really enjoyed enjoyed. We would love to do this again....</t>
+  </si>
+  <si>
+    <t>review_f9cdb9eca2ee3cc58a058227 :: Even on an overcast day, the views were stunning. My hubby said I couldn't stop smiling. I was mesmerized. My first helicopter ride and it was fantastic. Pilot Shawn was just infor...</t>
+  </si>
+  <si>
+    <t>review_a9dd2820ca31d2ba3296a18c :: Friends and I looked into a flight seeing tour of Denali and the glaciers and we were not dissapointed. The pilot, Jeff, was a great tour guide. He was very informative and managed...</t>
+  </si>
+  <si>
+    <t>review_839e0560238a0af9aac3153f :: I am a terrible flier. As in PETRIFIED.  Somehow, though, this clean, well kept little dock caught my eye as my husband and I drove into Talkeetna for one overnight. Despite my fea...</t>
   </si>
   <si>
     <t>review_5d3aa0665da02a18fbb9d035 :: Our experience was awesome! 
 They waterproof shoes that slipped over our own boots for the glacier landing. Our experience was during Covid-19 and the whole staff took extra preca...</t>
   </si>
   <si>
-    <t>review_a9dd2820ca31d2ba3296a18c :: Friends and I looked into a flight seeing tour of Denali and the glaciers and we were not dissapointed. The pilot, Jeff, was a great tour guide. He was very informative and managed...</t>
-  </si>
-  <si>
-    <t>review_839e0560238a0af9aac3153f :: I am a terrible flier. As in PETRIFIED.  Somehow, though, this clean, well kept little dock caught my eye as my husband and I drove into Talkeetna for one overnight. Despite my fea...</t>
-  </si>
-  <si>
-    <t>review_b1f4591ba3fe0c7697725cd4 :: Just an incredible time and an experience to be cherished. We had a lot of fun and really enjoyed enjoyed. We would love to do this again....</t>
-  </si>
-  <si>
-    <t>review_f9cdb9eca2ee3cc58a058227 :: Even on an overcast day, the views were stunning. My hubby said I couldn't stop smiling. I was mesmerized. My first helicopter ride and it was fantastic. Pilot Shawn was just infor...</t>
-  </si>
-  <si>
     <t>review_0906e867106940cb3451f5d4 :: If you have a chance to go, definitely do it. I was able to do the glacier landing. Our weather that day was perfect. It is amazing to fly around the range and a great way to get a...</t>
   </si>
   <si>
@@ -621,79 +639,61 @@
     <t>review_b08abf39f399085373741cfc :: This was a 12 hour adventure to remember - it started with a flight over the Grand Canyon to Page, Arizona where we were then taken to the amazing slot canyons of Antelope Canyon v...</t>
   </si>
   <si>
+    <t>review_5e1ada412e6d27e61871d3d2 :: My husband and I booked the Canyon Spirit, 45-50min tour with Maverick Helicopters as part of a 3 week tour around the west of America. We booked it online a month before we went t...</t>
+  </si>
+  <si>
+    <t>review_34b482736330103710d534dd :: Joe, the pilot, was not just knowledgable and interesting, he put us all at ease with clear safety instructions,  very obvious attention to his task, and some needed comedic relief...</t>
+  </si>
+  <si>
+    <t>review_d5b6da22fea5e1d569198664 :: I am recently retired, and a trip to Alaska was one of my 'bucket list' destinations.  This flightseeing tour over Denali was the crown jewel of the trip.  Truly amazing, and a lif...</t>
+  </si>
+  <si>
+    <t>review_106dc23da845ce9e90ce924e :: This is the third time I have taken this trip and it never ceases to amaze. You cannot appreciate the Grand Canyon from just seeing pictures and flying over and through. It gives a...</t>
+  </si>
+  <si>
     <t>review_9d1f6ad84d606ddca5e4e615 :: This flight was great and the narration was really very interesting and the landing was just sublime...</t>
   </si>
   <si>
-    <t>review_106dc23da845ce9e90ce924e :: This is the third time I have taken this trip and it never ceases to amaze. You cannot appreciate the Grand Canyon from just seeing pictures and flying over and through. It gives a...</t>
-  </si>
-  <si>
-    <t>review_5e1ada412e6d27e61871d3d2 :: My husband and I booked the Canyon Spirit, 45-50min tour with Maverick Helicopters as part of a 3 week tour around the west of America. We booked it online a month before we went t...</t>
-  </si>
-  <si>
-    <t>review_34b482736330103710d534dd :: Joe, the pilot, was not just knowledgable and interesting, he put us all at ease with clear safety instructions,  very obvious attention to his task, and some needed comedic relief...</t>
-  </si>
-  <si>
-    <t>review_d5b6da22fea5e1d569198664 :: I am recently retired, and a trip to Alaska was one of my 'bucket list' destinations.  This flightseeing tour over Denali was the crown jewel of the trip.  Truly amazing, and a lif...</t>
+    <t>review_23dd8ca7ccb1504a0fdd0abe :: Having made a reservation to do a flightseeing trip months before we arrived in Talkeetna, I had the very good fortunate to have the sun shining throughout this spectacular trip. M...</t>
+  </si>
+  <si>
+    <t>review_a20afea77622e7f2a696a5b8 :: Friday Harbor seaplanes was an exceptional way to travel into Friday Harbor.  They were friendly, helpful and made the whole experience great.  Getting to FH can be stressful and t...</t>
+  </si>
+  <si>
+    <t>review_a6393fcd3d1377ade8951ba7 :: Our trip was in May 2022. We had a blast. The pilot was knowledgeable and fun. My husband hates flying, especially small planes, but he'd do it again. We plan to book with K2 again...</t>
+  </si>
+  <si>
+    <t>review_e07d338aaa29596c79153eae :: Denali was not an option the day we went because of bad weather so they offered us another tour.  We had a wonderful pilot and got to see a lot.  I was in the co-pilot seat which w...</t>
+  </si>
+  <si>
+    <t>review_182483adf502c67405c09314 :: Our second time with our pilot, and as amazing as the first time. We will do it a third and hopefully a fourth too. Exhilerating...</t>
+  </si>
+  <si>
+    <t>review_c542b91f8f33b62598c7e8e7 :: The whole experience was fabulous from the convenience of short notice booking to the easy check in and ultimately with the flight and our pilot! The facility is welcoming and the ...</t>
+  </si>
+  <si>
+    <t>review_5fe9fad9238c2de93e358451 :: I had a "reservation" to fly, but waited over a hour. I saw lightening and storm clouds- I was told by pilot that it was a small cell that we'd fly around. IMMEDIATELY after takeof...</t>
+  </si>
+  <si>
+    <t>review_1414273dd7063c526a44d117 :: This was one of lifetime plane trip realy memorable. I simply envy pilots they get to do this and get paid for it. Just seeing the wonderful mountain range up close is breathtaking...</t>
+  </si>
+  <si>
+    <t>review_0e57afe5271794777fc522b8 :: The tour was wonderful ! what a pity that no comment is in another language than english and that the pilot doesn't care if the passengers understand or not what he says during the...</t>
+  </si>
+  <si>
+    <t>review_805ef5f7c1f0df545b37c9b0 :: Isaac was an excellent pilot and very thorough in explaining island sites, and comforting some first time jitters about flying in a small plane. Loved that it was just me, my husba...</t>
   </si>
   <si>
     <t>review_5035b0fc89c249531e5a177f :: My family and I toured with K2 on a day that didn't have great weather. We were supposed to have a flightseeing tour and glacier landing at 1 pm, but because the weather was poor, ...</t>
   </si>
   <si>
-    <t>review_805ef5f7c1f0df545b37c9b0 :: Isaac was an excellent pilot and very thorough in explaining island sites, and comforting some first time jitters about flying in a small plane. Loved that it was just me, my husba...</t>
-  </si>
-  <si>
-    <t>review_0e57afe5271794777fc522b8 :: The tour was wonderful ! what a pity that no comment is in another language than english and that the pilot doesn't care if the passengers understand or not what he says during the...</t>
-  </si>
-  <si>
-    <t>review_1414273dd7063c526a44d117 :: This was one of lifetime plane trip realy memorable. I simply envy pilots they get to do this and get paid for it. Just seeing the wonderful mountain range up close is breathtaking...</t>
-  </si>
-  <si>
-    <t>review_5fe9fad9238c2de93e358451 :: I had a "reservation" to fly, but waited over a hour. I saw lightening and storm clouds- I was told by pilot that it was a small cell that we'd fly around. IMMEDIATELY after takeof...</t>
-  </si>
-  <si>
-    <t>review_23dd8ca7ccb1504a0fdd0abe :: Having made a reservation to do a flightseeing trip months before we arrived in Talkeetna, I had the very good fortunate to have the sun shining throughout this spectacular trip. M...</t>
-  </si>
-  <si>
-    <t>review_182483adf502c67405c09314 :: Our second time with our pilot, and as amazing as the first time. We will do it a third and hopefully a fourth too. Exhilerating...</t>
-  </si>
-  <si>
-    <t>review_c542b91f8f33b62598c7e8e7 :: The whole experience was fabulous from the convenience of short notice booking to the easy check in and ultimately with the flight and our pilot! The facility is welcoming and the ...</t>
-  </si>
-  <si>
-    <t>review_e07d338aaa29596c79153eae :: Denali was not an option the day we went because of bad weather so they offered us another tour.  We had a wonderful pilot and got to see a lot.  I was in the co-pilot seat which w...</t>
-  </si>
-  <si>
-    <t>review_a6393fcd3d1377ade8951ba7 :: Our trip was in May 2022. We had a blast. The pilot was knowledgeable and fun. My husband hates flying, especially small planes, but he'd do it again. We plan to book with K2 again...</t>
-  </si>
-  <si>
-    <t>review_a20afea77622e7f2a696a5b8 :: Friday Harbor seaplanes was an exceptional way to travel into Friday Harbor.  They were friendly, helpful and made the whole experience great.  Getting to FH can be stressful and t...</t>
-  </si>
-  <si>
-    <t>review_2ced2be9a338446e48906797 :: "Best hour of my life"--or at least that's how my daughter (not a little kid, but rather a highly accomplished and well travelled professional) described it.  While I trust her exc...</t>
-  </si>
-  <si>
-    <t>review_3586d47de5356ce1da25e642 :: Everything about K2 inspires confidence, which is essential if you're planning to ride a small plane up thousands of feet for a closer look at mountains and glaciers. The planes ar...</t>
-  </si>
-  <si>
-    <t>review_721ad19aff869f0d170db596 :: Our five island tour started out overlooking West Maui and then we set across the channel to the Molokai sea cliffs...just beautiful.  We then circled around for a 180-degree view ...</t>
-  </si>
-  <si>
-    <t>review_690cc278985c56f33f02481e :: We booked this trip through our Disney cruise.  The day we went the weather was beautiful.  But Ketchikan is in an artic rain forest so I understand these tours are often cancelled...</t>
-  </si>
-  <si>
-    <t>review_1dd85bf8878c66fc279b0b60 :: We travelled from Scotland to the USA to ride down the famous Route 66. One of my most anticipated stops was to see the Grand Canyon. But it was also one of my most dreaded... perh...</t>
-  </si>
-  <si>
-    <t>review_74b3950bfc8651a0c192c5f7 :: From the moment we took off to the moment we landed back at the airport we were all spellbound!  The ride was amazing and I would highly recommend it.  We landed on Ruth Glacier an...</t>
-  </si>
-  <si>
     <t>review_e9b2f31c772c2b7cb28b91a6 :: I am a very anxious flyer but wanted to see the Na Pali coast badly so I booked a private tour in the Cessna.  Bruce was our pilot and he was excellent at giving the tour and makin...</t>
   </si>
   <si>
-    <t>review_e0e8c4638a54285feff0cfbc :: CHEAPER IF BOOKED DIRECTLY, but if there are scheduling problems with your cruise line and you're late, it's better to have booked thru the cruise line.  There is an option especia...</t>
-  </si>
-  <si>
-    <t>review_6a2174ace00b3c34805ab86a :: When you live on Kauai, you have the ability to pick and choose. One of our best choices (other than making the decision to move here) was picking to take a Wings Over Kauai flight...</t>
+    <t>review_e64fadc568774df30ea12ccb :: Our pilot, Rosemarie, provided a wonderful flight and narration.   She was consistently focused on meeting our needs, answering questions with insightful responses, and proactively...</t>
+  </si>
+  <si>
+    <t>review_e6cf6dd7ddebb8be79394b82 :: This is one of the most amazing trips we have ever been on. The scenery was breathtaking. Great ambience and very tranquil to see the view from the plane. Thank you for such a grea...</t>
   </si>
   <si>
     <t>review_a1479d7709ac1f0657a6be34 :: I was a little nervous about this-especially since I am 62 and my husband is 73-
@@ -701,63 +701,87 @@
 From the...</t>
   </si>
   <si>
-    <t>review_e6cf6dd7ddebb8be79394b82 :: This is one of the most amazing trips we have ever been on. The scenery was breathtaking. Great ambience and very tranquil to see the view from the plane. Thank you for such a grea...</t>
-  </si>
-  <si>
-    <t>review_61a9d3d1fdbcd064bf4345ca :: We had an amazing Denali experience with Matt as our wonderful pilot!  Staff at the facility were very helpful and friendly making sure we knew what to do prior to boarding aircraf...</t>
-  </si>
-  <si>
-    <t>review_3e78e4ee92bd76c4cb21392e :: There were 8 of us on the plane. We all had window seats so great viewing. They provide an automated narration via headphones which is interesting  and informative. We were a group...</t>
-  </si>
-  <si>
-    <t>review_afef78fc89e72cc13bcb4c60 :: When we arrived in Ketchikan on Tuesday, June 23, 2015, it was a beautiful day so we decided to book a seaplane excursion of the Misty Fjords.  We ended up at Taquan Air and everyo...</t>
-  </si>
-  <si>
-    <t>review_103f4440d6a6486ab6782f17 :: Taquan is situated across the channel from the Ketchikan Airport, a 5 minute ride on the ferry. With wheeled luggage an easy hop from the terminal. No taxi required. I showed up an...</t>
-  </si>
-  <si>
-    <t>review_4a582265ded51274209a4ffc :: The Denali flightseeing adventure was oustanding. Beautiful day, 10 passenger plane, smooth flight, great pilot and the most unbelievable views of the mountain and glaciers. In 40 ...</t>
-  </si>
-  <si>
-    <t>review_539ab35db100ef8bcf0f37b8 :: I'm older (60s) my friend is OLDER (72) and yet we really wanted to go--K2 has great staff, so kind and helpful in many ways. The biggest part of the trip is in the plane looking o...</t>
+    <t>review_6a2174ace00b3c34805ab86a :: When you live on Kauai, you have the ability to pick and choose. One of our best choices (other than making the decision to move here) was picking to take a Wings Over Kauai flight...</t>
+  </si>
+  <si>
+    <t>review_e0e8c4638a54285feff0cfbc :: CHEAPER IF BOOKED DIRECTLY, but if there are scheduling problems with your cruise line and you're late, it's better to have booked thru the cruise line.  There is an option especia...</t>
+  </si>
+  <si>
+    <t>review_2ced2be9a338446e48906797 :: "Best hour of my life"--or at least that's how my daughter (not a little kid, but rather a highly accomplished and well travelled professional) described it.  While I trust her exc...</t>
+  </si>
+  <si>
+    <t>review_74b3950bfc8651a0c192c5f7 :: From the moment we took off to the moment we landed back at the airport we were all spellbound!  The ride was amazing and I would highly recommend it.  We landed on Ruth Glacier an...</t>
+  </si>
+  <si>
+    <t>review_690cc278985c56f33f02481e :: We booked this trip through our Disney cruise.  The day we went the weather was beautiful.  But Ketchikan is in an artic rain forest so I understand these tours are often cancelled...</t>
+  </si>
+  <si>
+    <t>review_721ad19aff869f0d170db596 :: Our five island tour started out overlooking West Maui and then we set across the channel to the Molokai sea cliffs...just beautiful.  We then circled around for a 180-degree view ...</t>
+  </si>
+  <si>
+    <t>review_3586d47de5356ce1da25e642 :: Everything about K2 inspires confidence, which is essential if you're planning to ride a small plane up thousands of feet for a closer look at mountains and glaciers. The planes ar...</t>
+  </si>
+  <si>
+    <t>review_1dd85bf8878c66fc279b0b60 :: We travelled from Scotland to the USA to ride down the famous Route 66. One of my most anticipated stops was to see the Grand Canyon. But it was also one of my most dreaded... perh...</t>
+  </si>
+  <si>
+    <t>review_fd2e1ec4090146c614767640 :: I don't like to fly in small planes or helicopters (fear of heights!) - but this was awesome! Bruce gave us a special glimpse of the beautiful Kauai, and his information and commen...</t>
+  </si>
+  <si>
+    <t>review_b7f01c12e058877205debe1a :: This was a great experience from start to finish, starting with quick responses to initial enquiries, preflight contacts and information, safety briefing and the engagement of an e...</t>
+  </si>
+  <si>
+    <t>review_f630d22ae67bb1aea6cde23c :: Steve was great captain. We had 9 passenger. Didn’t have to pay extra $15 for window seat. If you end up going into larger flight you will be asked if you want to. 
+Ps. Thank you S...</t>
+  </si>
+  <si>
+    <t>review_9cc699fcb8b3d3fab878cc9f :: I'm conflicted as to how to review Westwind as we had two different planes for our group of 16 family and friends (ages ranging from 25 - 60) who had completely different experienc...</t>
+  </si>
+  <si>
+    <t>review_a3f8d14b3c831abdc1614668 :: With a young family we found our options for aerial tours was limited as most helicopter tours would not take a child under 2 years.  While we didn't take our young child on the to...</t>
+  </si>
+  <si>
+    <t>review_a485c5e820c7e55c86de9a0b :: We decided on a whim to do a plane tour of Maui. WOW did we pick the right guy. The plane was as smooth as the operator. Absolutely flawless. We have done a ton of things so far on...</t>
+  </si>
+  <si>
+    <t>review_6ef8c900520da66d485e0c4e :: It was a wonderful experience. Thank you! Super great. Yay. Would do again. Beautiful. Nice guy. Good company....</t>
+  </si>
+  <si>
+    <t>review_ff7695c5a050f9db720f89a9 :: This company at least needs to train there employees to have some compassion or emotion for a helicopter ride that needs to be cancelled because of the weather (high winds).  Yes, ...</t>
+  </si>
+  <si>
+    <t>review_8bc91ab41a9ca49ce95dc25c :: I was overjoyed by this seaplane experience!  Breathtaking views, some of the prettiest scenery I have ever seen.  Our pilot, Shane, was very engaging and informative.  The landing...</t>
+  </si>
+  <si>
+    <t>review_be756d082c9857ee2d7f2a8b :: Had a blast! Eric was great and friendly, we had an awesome time flying over Volcanoes National Park and taking a pit stop in Hilo for lunch. 10/10 would definitely recommend! I’ve...</t>
+  </si>
+  <si>
+    <t>review_bf34bf6197d91084faf96975 :: Whatever you do, don't miss this experience when visiting Kauai.  Our family of four were the only ones on the plane as we booked a private charter, so it was very personal and we ...</t>
+  </si>
+  <si>
+    <t>review_84a78a9d4bfb31d92af294ad :: I can't say enough positive things about this amazing experience. It was worth every penny and then some. Will(bur?) was an excellent pilot and a downright excellent human. He was ...</t>
   </si>
   <si>
     <t>review_9502735c5977685b4e9511be :: Nice way to see beautiful Kauai. Glad we chose these guys, the whole team was great. We will recommend this to our friends.
 Our pilot, Josh was amazing. Friendly, experienced and ...</t>
   </si>
   <si>
-    <t>review_84a78a9d4bfb31d92af294ad :: I can't say enough positive things about this amazing experience. It was worth every penny and then some. Will(bur?) was an excellent pilot and a downright excellent human. He was ...</t>
-  </si>
-  <si>
-    <t>review_be756d082c9857ee2d7f2a8b :: Had a blast! Eric was great and friendly, we had an awesome time flying over Volcanoes National Park and taking a pit stop in Hilo for lunch. 10/10 would definitely recommend! I’ve...</t>
-  </si>
-  <si>
-    <t>review_bf34bf6197d91084faf96975 :: Whatever you do, don't miss this experience when visiting Kauai.  Our family of four were the only ones on the plane as we booked a private charter, so it was very personal and we ...</t>
-  </si>
-  <si>
-    <t>review_fd2e1ec4090146c614767640 :: I don't like to fly in small planes or helicopters (fear of heights!) - but this was awesome! Bruce gave us a special glimpse of the beautiful Kauai, and his information and commen...</t>
-  </si>
-  <si>
-    <t>review_8bc91ab41a9ca49ce95dc25c :: I was overjoyed by this seaplane experience!  Breathtaking views, some of the prettiest scenery I have ever seen.  Our pilot, Shane, was very engaging and informative.  The landing...</t>
-  </si>
-  <si>
-    <t>review_ff7695c5a050f9db720f89a9 :: This company at least needs to train there employees to have some compassion or emotion for a helicopter ride that needs to be cancelled because of the weather (high winds).  Yes, ...</t>
-  </si>
-  <si>
-    <t>review_6ef8c900520da66d485e0c4e :: It was a wonderful experience. Thank you! Super great. Yay. Would do again. Beautiful. Nice guy. Good company....</t>
-  </si>
-  <si>
-    <t>review_a485c5e820c7e55c86de9a0b :: We decided on a whim to do a plane tour of Maui. WOW did we pick the right guy. The plane was as smooth as the operator. Absolutely flawless. We have done a ton of things so far on...</t>
-  </si>
-  <si>
-    <t>review_a3f8d14b3c831abdc1614668 :: With a young family we found our options for aerial tours was limited as most helicopter tours would not take a child under 2 years.  While we didn't take our young child on the to...</t>
-  </si>
-  <si>
-    <t>review_9cc699fcb8b3d3fab878cc9f :: I'm conflicted as to how to review Westwind as we had two different planes for our group of 16 family and friends (ages ranging from 25 - 60) who had completely different experienc...</t>
-  </si>
-  <si>
-    <t>review_f630d22ae67bb1aea6cde23c :: Steve was great captain. We had 9 passenger. Didn’t have to pay extra $15 for window seat. If you end up going into larger flight you will be asked if you want to. 
-Ps. Thank you S...</t>
+    <t>review_539ab35db100ef8bcf0f37b8 :: I'm older (60s) my friend is OLDER (72) and yet we really wanted to go--K2 has great staff, so kind and helpful in many ways. The biggest part of the trip is in the plane looking o...</t>
+  </si>
+  <si>
+    <t>review_4a582265ded51274209a4ffc :: The Denali flightseeing adventure was oustanding. Beautiful day, 10 passenger plane, smooth flight, great pilot and the most unbelievable views of the mountain and glaciers. In 40 ...</t>
+  </si>
+  <si>
+    <t>review_103f4440d6a6486ab6782f17 :: Taquan is situated across the channel from the Ketchikan Airport, a 5 minute ride on the ferry. With wheeled luggage an easy hop from the terminal. No taxi required. I showed up an...</t>
+  </si>
+  <si>
+    <t>review_afef78fc89e72cc13bcb4c60 :: When we arrived in Ketchikan on Tuesday, June 23, 2015, it was a beautiful day so we decided to book a seaplane excursion of the Misty Fjords.  We ended up at Taquan Air and everyo...</t>
+  </si>
+  <si>
+    <t>review_3e78e4ee92bd76c4cb21392e :: There were 8 of us on the plane. We all had window seats so great viewing. They provide an automated narration via headphones which is interesting  and informative. We were a group...</t>
+  </si>
+  <si>
+    <t>review_61a9d3d1fdbcd064bf4345ca :: We had an amazing Denali experience with Matt as our wonderful pilot!  Staff at the facility were very helpful and friendly making sure we knew what to do prior to boarding aircraf...</t>
   </si>
 </sst>
 </file>
@@ -1115,7 +1139,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1152,13 +1176,13 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F2">
         <v>42</v>
@@ -1167,7 +1191,7 @@
         <v>39</v>
       </c>
       <c r="H2" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1175,16 +1199,16 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D3" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F3">
         <v>37</v>
@@ -1193,7 +1217,7 @@
         <v>37</v>
       </c>
       <c r="H3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1204,13 +1228,13 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D4" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E4" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="F4">
         <v>28</v>
@@ -1219,7 +1243,7 @@
         <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1230,13 +1254,13 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D5" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="E5" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F5">
         <v>20</v>
@@ -1245,7 +1269,7 @@
         <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1256,13 +1280,13 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D6" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="E6" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F6">
         <v>16</v>
@@ -1271,7 +1295,7 @@
         <v>16</v>
       </c>
       <c r="H6" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1282,13 +1306,13 @@
         <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D7" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E7" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F7">
         <v>15</v>
@@ -1297,7 +1321,7 @@
         <v>15</v>
       </c>
       <c r="H7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1308,13 +1332,13 @@
         <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D8" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="E8" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F8">
         <v>10</v>
@@ -1323,7 +1347,7 @@
         <v>9</v>
       </c>
       <c r="H8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1331,16 +1355,16 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D9" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E9" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F9">
         <v>8</v>
@@ -1349,7 +1373,7 @@
         <v>8</v>
       </c>
       <c r="H9" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1357,25 +1381,25 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D10" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="E10" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F10">
         <v>8</v>
       </c>
       <c r="G10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H10" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1383,25 +1407,25 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>75</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D11" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="E11" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F11">
         <v>8</v>
       </c>
       <c r="G11">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H11" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1409,16 +1433,16 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D12" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="E12" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F12">
         <v>8</v>
@@ -1427,7 +1451,7 @@
         <v>8</v>
       </c>
       <c r="H12" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1438,13 +1462,13 @@
         <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D13" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="E13" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F13">
         <v>8</v>
@@ -1453,7 +1477,7 @@
         <v>8</v>
       </c>
       <c r="H13" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1464,13 +1488,13 @@
         <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D14" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="E14" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F14">
         <v>7</v>
@@ -1479,7 +1503,7 @@
         <v>7</v>
       </c>
       <c r="H14" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1487,16 +1511,16 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C15" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D15" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E15" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="F15">
         <v>7</v>
@@ -1505,7 +1529,7 @@
         <v>7</v>
       </c>
       <c r="H15" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1516,13 +1540,13 @@
         <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D16" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E16" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F16">
         <v>7</v>
@@ -1531,7 +1555,7 @@
         <v>6</v>
       </c>
       <c r="H16" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1542,13 +1566,13 @@
         <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D17" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="E17" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F17">
         <v>6</v>
@@ -1557,7 +1581,7 @@
         <v>6</v>
       </c>
       <c r="H17" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1568,22 +1592,22 @@
         <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D18" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="E18" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F18">
         <v>6</v>
       </c>
       <c r="G18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H18" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1594,13 +1618,13 @@
         <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D19" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="E19" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F19">
         <v>6</v>
@@ -1609,7 +1633,7 @@
         <v>6</v>
       </c>
       <c r="H19" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1620,22 +1644,22 @@
         <v>26</v>
       </c>
       <c r="C20" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D20" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E20" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F20">
         <v>6</v>
       </c>
       <c r="G20">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H20" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1646,13 +1670,13 @@
         <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D21" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="E21" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F21">
         <v>6</v>
@@ -1661,7 +1685,7 @@
         <v>6</v>
       </c>
       <c r="H21" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1669,16 +1693,16 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D22" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E22" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F22">
         <v>5</v>
@@ -1687,7 +1711,7 @@
         <v>5</v>
       </c>
       <c r="H22" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1698,13 +1722,13 @@
         <v>29</v>
       </c>
       <c r="C23" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D23" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="E23" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F23">
         <v>5</v>
@@ -1713,7 +1737,7 @@
         <v>5</v>
       </c>
       <c r="H23" t="s">
-        <v>186</v>
+        <v>213</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1721,16 +1745,16 @@
         <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="C24" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D24" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="E24" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F24">
         <v>5</v>
@@ -1739,7 +1763,7 @@
         <v>5</v>
       </c>
       <c r="H24" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1750,13 +1774,13 @@
         <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D25" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E25" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -1765,7 +1789,7 @@
         <v>5</v>
       </c>
       <c r="H25" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1773,25 +1797,25 @@
         <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="C26" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D26" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E26" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F26">
         <v>5</v>
       </c>
       <c r="G26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H26" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1799,25 +1823,25 @@
         <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="C27" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D27" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="E27" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F27">
         <v>5</v>
       </c>
       <c r="G27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H27" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1825,16 +1849,16 @@
         <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C28" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E28" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F28">
         <v>5</v>
@@ -1843,7 +1867,7 @@
         <v>5</v>
       </c>
       <c r="H28" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1851,25 +1875,25 @@
         <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D29" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="E29" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F29">
         <v>5</v>
       </c>
       <c r="G29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H29" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1880,22 +1904,22 @@
         <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="E30" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F30">
         <v>5</v>
       </c>
       <c r="G30">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H30" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1906,13 +1930,13 @@
         <v>37</v>
       </c>
       <c r="C31" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D31" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="E31" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F31">
         <v>5</v>
@@ -1921,7 +1945,7 @@
         <v>5</v>
       </c>
       <c r="H31" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1929,16 +1953,16 @@
         <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D32" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="E32" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F32">
         <v>5</v>
@@ -1947,7 +1971,7 @@
         <v>5</v>
       </c>
       <c r="H32" t="s">
-        <v>215</v>
+        <v>192</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1958,13 +1982,13 @@
         <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D33" t="s">
-        <v>143</v>
+        <v>172</v>
       </c>
       <c r="E33" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F33">
         <v>5</v>
@@ -1973,7 +1997,7 @@
         <v>5</v>
       </c>
       <c r="H33" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -1981,25 +2005,25 @@
         <v>40</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D34" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="E34" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F34">
         <v>4</v>
       </c>
       <c r="G34">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H34" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2010,13 +2034,13 @@
         <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D35" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="E35" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F35">
         <v>4</v>
@@ -2025,7 +2049,7 @@
         <v>4</v>
       </c>
       <c r="H35" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2036,13 +2060,13 @@
         <v>42</v>
       </c>
       <c r="C36" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D36" t="s">
         <v>149</v>
       </c>
       <c r="E36" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F36">
         <v>4</v>
@@ -2051,7 +2075,7 @@
         <v>4</v>
       </c>
       <c r="H36" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2062,13 +2086,13 @@
         <v>43</v>
       </c>
       <c r="C37" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D37" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="E37" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F37">
         <v>4</v>
@@ -2077,7 +2101,7 @@
         <v>4</v>
       </c>
       <c r="H37" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2085,16 +2109,16 @@
         <v>44</v>
       </c>
       <c r="B38" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="C38" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E38" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F38">
         <v>4</v>
@@ -2103,7 +2127,7 @@
         <v>4</v>
       </c>
       <c r="H38" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2111,16 +2135,16 @@
         <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="C39" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D39" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="E39" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -2129,7 +2153,7 @@
         <v>4</v>
       </c>
       <c r="H39" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -2137,16 +2161,16 @@
         <v>46</v>
       </c>
       <c r="B40" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="C40" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D40" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="E40" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F40">
         <v>4</v>
@@ -2155,7 +2179,7 @@
         <v>4</v>
       </c>
       <c r="H40" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2166,22 +2190,22 @@
         <v>47</v>
       </c>
       <c r="C41" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D41" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="E41" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F41">
         <v>4</v>
       </c>
       <c r="G41">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H41" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -2189,16 +2213,16 @@
         <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="C42" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D42" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="E42" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F42">
         <v>4</v>
@@ -2207,7 +2231,7 @@
         <v>4</v>
       </c>
       <c r="H42" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2218,13 +2242,13 @@
         <v>49</v>
       </c>
       <c r="C43" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D43" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="E43" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F43">
         <v>4</v>
@@ -2233,7 +2257,7 @@
         <v>4</v>
       </c>
       <c r="H43" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2244,13 +2268,13 @@
         <v>50</v>
       </c>
       <c r="C44" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D44" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="E44" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F44">
         <v>4</v>
@@ -2259,7 +2283,7 @@
         <v>4</v>
       </c>
       <c r="H44" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2270,13 +2294,13 @@
         <v>51</v>
       </c>
       <c r="C45" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D45" t="s">
-        <v>143</v>
+        <v>177</v>
       </c>
       <c r="E45" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F45">
         <v>4</v>
@@ -2285,7 +2309,7 @@
         <v>4</v>
       </c>
       <c r="H45" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2293,25 +2317,25 @@
         <v>52</v>
       </c>
       <c r="B46" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="C46" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D46" t="s">
-        <v>158</v>
+        <v>178</v>
       </c>
       <c r="E46" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F46">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G46">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H46" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -2319,16 +2343,16 @@
         <v>53</v>
       </c>
       <c r="B47" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
       <c r="C47" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D47" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E47" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F47">
         <v>3</v>
@@ -2337,7 +2361,7 @@
         <v>3</v>
       </c>
       <c r="H47" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2348,13 +2372,13 @@
         <v>54</v>
       </c>
       <c r="C48" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D48" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="E48" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F48">
         <v>3</v>
@@ -2363,7 +2387,7 @@
         <v>3</v>
       </c>
       <c r="H48" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -2374,13 +2398,13 @@
         <v>55</v>
       </c>
       <c r="C49" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D49" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E49" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F49">
         <v>3</v>
@@ -2389,7 +2413,7 @@
         <v>3</v>
       </c>
       <c r="H49" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -2400,13 +2424,13 @@
         <v>56</v>
       </c>
       <c r="C50" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D50" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="E50" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F50">
         <v>3</v>
@@ -2415,7 +2439,7 @@
         <v>3</v>
       </c>
       <c r="H50" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2426,13 +2450,13 @@
         <v>57</v>
       </c>
       <c r="C51" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D51" t="s">
-        <v>154</v>
+        <v>181</v>
       </c>
       <c r="E51" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F51">
         <v>3</v>
@@ -2441,7 +2465,7 @@
         <v>3</v>
       </c>
       <c r="H51" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2449,16 +2473,16 @@
         <v>58</v>
       </c>
       <c r="B52" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="C52" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D52" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="E52" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F52">
         <v>3</v>
@@ -2467,7 +2491,7 @@
         <v>3</v>
       </c>
       <c r="H52" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -2478,13 +2502,13 @@
         <v>59</v>
       </c>
       <c r="C53" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D53" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="E53" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F53">
         <v>3</v>
@@ -2493,7 +2517,7 @@
         <v>3</v>
       </c>
       <c r="H53" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2504,13 +2528,13 @@
         <v>60</v>
       </c>
       <c r="C54" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D54" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E54" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F54">
         <v>3</v>
@@ -2519,7 +2543,7 @@
         <v>3</v>
       </c>
       <c r="H54" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2527,16 +2551,16 @@
         <v>61</v>
       </c>
       <c r="B55" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="C55" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D55" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="E55" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F55">
         <v>3</v>
@@ -2545,7 +2569,7 @@
         <v>3</v>
       </c>
       <c r="H55" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2553,16 +2577,16 @@
         <v>62</v>
       </c>
       <c r="B56" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="C56" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D56" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="E56" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F56">
         <v>3</v>
@@ -2571,7 +2595,7 @@
         <v>3</v>
       </c>
       <c r="H56" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -2579,16 +2603,16 @@
         <v>63</v>
       </c>
       <c r="B57" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="C57" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D57" t="s">
-        <v>145</v>
+        <v>176</v>
       </c>
       <c r="E57" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F57">
         <v>3</v>
@@ -2597,7 +2621,7 @@
         <v>3</v>
       </c>
       <c r="H57" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2608,13 +2632,13 @@
         <v>64</v>
       </c>
       <c r="C58" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D58" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="E58" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F58">
         <v>3</v>
@@ -2623,7 +2647,7 @@
         <v>3</v>
       </c>
       <c r="H58" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2631,16 +2655,16 @@
         <v>65</v>
       </c>
       <c r="B59" t="s">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="C59" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D59" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="E59" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F59">
         <v>3</v>
@@ -2649,7 +2673,7 @@
         <v>3</v>
       </c>
       <c r="H59" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2660,13 +2684,13 @@
         <v>66</v>
       </c>
       <c r="C60" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D60" t="s">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="E60" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F60">
         <v>3</v>
@@ -2675,7 +2699,7 @@
         <v>3</v>
       </c>
       <c r="H60" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -2686,13 +2710,13 @@
         <v>67</v>
       </c>
       <c r="C61" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D61" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="E61" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F61">
         <v>3</v>
@@ -2701,7 +2725,7 @@
         <v>3</v>
       </c>
       <c r="H61" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -2712,13 +2736,13 @@
         <v>68</v>
       </c>
       <c r="C62" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D62" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="E62" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F62">
         <v>3</v>
@@ -2727,7 +2751,7 @@
         <v>3</v>
       </c>
       <c r="H62" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -2738,13 +2762,13 @@
         <v>69</v>
       </c>
       <c r="C63" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D63" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="E63" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F63">
         <v>3</v>
@@ -2753,7 +2777,85 @@
         <v>3</v>
       </c>
       <c r="H63" t="s">
-        <v>245</v>
+        <v>251</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64" t="s">
+        <v>70</v>
+      </c>
+      <c r="B64" t="s">
+        <v>70</v>
+      </c>
+      <c r="C64" t="s">
+        <v>146</v>
+      </c>
+      <c r="D64" t="s">
+        <v>189</v>
+      </c>
+      <c r="E64" t="s">
+        <v>190</v>
+      </c>
+      <c r="F64">
+        <v>3</v>
+      </c>
+      <c r="G64">
+        <v>3</v>
+      </c>
+      <c r="H64" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" t="s">
+        <v>71</v>
+      </c>
+      <c r="B65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C65" t="s">
+        <v>147</v>
+      </c>
+      <c r="D65" t="s">
+        <v>172</v>
+      </c>
+      <c r="E65" t="s">
+        <v>190</v>
+      </c>
+      <c r="F65">
+        <v>3</v>
+      </c>
+      <c r="G65">
+        <v>3</v>
+      </c>
+      <c r="H65" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" t="s">
+        <v>72</v>
+      </c>
+      <c r="B66" t="s">
+        <v>72</v>
+      </c>
+      <c r="C66" t="s">
+        <v>148</v>
+      </c>
+      <c r="D66" t="s">
+        <v>178</v>
+      </c>
+      <c r="E66" t="s">
+        <v>191</v>
+      </c>
+      <c r="F66">
+        <v>3</v>
+      </c>
+      <c r="G66">
+        <v>3</v>
+      </c>
+      <c r="H66" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ai): purge interjection yay from clean emotion lexicons
</commit_message>
<xml_diff>
--- a/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
+++ b/data/derived_outputs/stage_final/clean_new_emotion_words_18901.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="250">
   <si>
     <t>word</t>
   </si>
@@ -193,9 +193,6 @@
     <t>compassionate</t>
   </si>
   <si>
-    <t>yay</t>
-  </si>
-  <si>
     <t>compassion</t>
   </si>
   <si>
@@ -421,9 +418,6 @@
     <t>富有同理心体贴的</t>
   </si>
   <si>
-    <t>欢呼太棒了（情绪感叹）</t>
-  </si>
-  <si>
     <t>同理心 / 关切</t>
   </si>
   <si>
@@ -563,9 +557,6 @@
   </si>
   <si>
     <t>Compassion</t>
-  </si>
-  <si>
-    <t>Joy / Excitement</t>
   </si>
   <si>
     <t>Regret / Guilt</t>
@@ -742,9 +733,6 @@
   </si>
   <si>
     <t>review_a485c5e820c7e55c86de9a0b :: We decided on a whim to do a plane tour of Maui. WOW did we pick the right guy. The plane was as smooth as the operator. Absolutely flawless. We have done a ton of things so far on...</t>
-  </si>
-  <si>
-    <t>review_6ef8c900520da66d485e0c4e :: It was a wonderful experience. Thank you! Super great. Yay. Would do again. Beautiful. Nice guy. Good company....</t>
   </si>
   <si>
     <t>review_ff7695c5a050f9db720f89a9 :: This company at least needs to train there employees to have some compassion or emotion for a helicopter ride that needs to be cancelled because of the weather (high winds).  Yes, ...</t>
@@ -1139,7 +1127,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1176,13 +1164,13 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F2">
         <v>42</v>
@@ -1191,7 +1179,7 @@
         <v>39</v>
       </c>
       <c r="H2" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1199,16 +1187,16 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E3" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F3">
         <v>37</v>
@@ -1217,7 +1205,7 @@
         <v>37</v>
       </c>
       <c r="H3" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1228,13 +1216,13 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E4" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F4">
         <v>28</v>
@@ -1243,7 +1231,7 @@
         <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1254,13 +1242,13 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E5" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F5">
         <v>20</v>
@@ -1269,7 +1257,7 @@
         <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1280,13 +1268,13 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D6" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E6" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F6">
         <v>16</v>
@@ -1295,7 +1283,7 @@
         <v>16</v>
       </c>
       <c r="H6" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1306,13 +1294,13 @@
         <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E7" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F7">
         <v>15</v>
@@ -1321,7 +1309,7 @@
         <v>15</v>
       </c>
       <c r="H7" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1332,13 +1320,13 @@
         <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E8" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F8">
         <v>10</v>
@@ -1347,7 +1335,7 @@
         <v>9</v>
       </c>
       <c r="H8" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1355,16 +1343,16 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E9" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F9">
         <v>8</v>
@@ -1373,7 +1361,7 @@
         <v>8</v>
       </c>
       <c r="H9" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1384,13 +1372,13 @@
         <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E10" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F10">
         <v>8</v>
@@ -1399,7 +1387,7 @@
         <v>8</v>
       </c>
       <c r="H10" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1407,16 +1395,16 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E11" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F11">
         <v>8</v>
@@ -1425,7 +1413,7 @@
         <v>7</v>
       </c>
       <c r="H11" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1436,13 +1424,13 @@
         <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E12" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F12">
         <v>8</v>
@@ -1451,7 +1439,7 @@
         <v>8</v>
       </c>
       <c r="H12" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1462,13 +1450,13 @@
         <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D13" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E13" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F13">
         <v>8</v>
@@ -1477,7 +1465,7 @@
         <v>8</v>
       </c>
       <c r="H13" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1488,13 +1476,13 @@
         <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D14" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E14" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F14">
         <v>7</v>
@@ -1503,7 +1491,7 @@
         <v>7</v>
       </c>
       <c r="H14" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1511,16 +1499,16 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E15" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F15">
         <v>7</v>
@@ -1529,7 +1517,7 @@
         <v>7</v>
       </c>
       <c r="H15" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1540,13 +1528,13 @@
         <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E16" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F16">
         <v>7</v>
@@ -1555,7 +1543,7 @@
         <v>6</v>
       </c>
       <c r="H16" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1566,13 +1554,13 @@
         <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D17" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E17" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F17">
         <v>6</v>
@@ -1581,7 +1569,7 @@
         <v>6</v>
       </c>
       <c r="H17" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1592,13 +1580,13 @@
         <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D18" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E18" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F18">
         <v>6</v>
@@ -1607,7 +1595,7 @@
         <v>6</v>
       </c>
       <c r="H18" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1618,13 +1606,13 @@
         <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E19" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F19">
         <v>6</v>
@@ -1633,7 +1621,7 @@
         <v>6</v>
       </c>
       <c r="H19" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1644,13 +1632,13 @@
         <v>26</v>
       </c>
       <c r="C20" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D20" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E20" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F20">
         <v>6</v>
@@ -1659,7 +1647,7 @@
         <v>5</v>
       </c>
       <c r="H20" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1670,13 +1658,13 @@
         <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D21" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E21" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F21">
         <v>6</v>
@@ -1685,7 +1673,7 @@
         <v>6</v>
       </c>
       <c r="H21" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1693,16 +1681,16 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D22" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E22" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F22">
         <v>5</v>
@@ -1711,7 +1699,7 @@
         <v>5</v>
       </c>
       <c r="H22" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1722,13 +1710,13 @@
         <v>29</v>
       </c>
       <c r="C23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D23" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E23" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F23">
         <v>5</v>
@@ -1737,7 +1725,7 @@
         <v>5</v>
       </c>
       <c r="H23" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1745,16 +1733,16 @@
         <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D24" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E24" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F24">
         <v>5</v>
@@ -1763,7 +1751,7 @@
         <v>5</v>
       </c>
       <c r="H24" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1774,13 +1762,13 @@
         <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D25" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E25" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -1789,7 +1777,7 @@
         <v>5</v>
       </c>
       <c r="H25" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1797,16 +1785,16 @@
         <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D26" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E26" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F26">
         <v>5</v>
@@ -1815,7 +1803,7 @@
         <v>4</v>
       </c>
       <c r="H26" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1826,13 +1814,13 @@
         <v>33</v>
       </c>
       <c r="C27" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D27" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E27" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F27">
         <v>5</v>
@@ -1841,7 +1829,7 @@
         <v>4</v>
       </c>
       <c r="H27" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1849,16 +1837,16 @@
         <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C28" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D28" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E28" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F28">
         <v>5</v>
@@ -1867,7 +1855,7 @@
         <v>5</v>
       </c>
       <c r="H28" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1878,13 +1866,13 @@
         <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D29" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E29" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F29">
         <v>5</v>
@@ -1893,7 +1881,7 @@
         <v>5</v>
       </c>
       <c r="H29" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1904,13 +1892,13 @@
         <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D30" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E30" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F30">
         <v>5</v>
@@ -1919,7 +1907,7 @@
         <v>5</v>
       </c>
       <c r="H30" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1930,13 +1918,13 @@
         <v>37</v>
       </c>
       <c r="C31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D31" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E31" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F31">
         <v>5</v>
@@ -1945,7 +1933,7 @@
         <v>5</v>
       </c>
       <c r="H31" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1956,13 +1944,13 @@
         <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D32" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E32" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F32">
         <v>5</v>
@@ -1971,7 +1959,7 @@
         <v>5</v>
       </c>
       <c r="H32" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1982,13 +1970,13 @@
         <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D33" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E33" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F33">
         <v>5</v>
@@ -1997,7 +1985,7 @@
         <v>5</v>
       </c>
       <c r="H33" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -2008,13 +1996,13 @@
         <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D34" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E34" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F34">
         <v>4</v>
@@ -2023,7 +2011,7 @@
         <v>3</v>
       </c>
       <c r="H34" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2034,13 +2022,13 @@
         <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D35" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E35" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F35">
         <v>4</v>
@@ -2049,7 +2037,7 @@
         <v>4</v>
       </c>
       <c r="H35" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2060,13 +2048,13 @@
         <v>42</v>
       </c>
       <c r="C36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D36" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E36" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F36">
         <v>4</v>
@@ -2075,7 +2063,7 @@
         <v>4</v>
       </c>
       <c r="H36" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2086,13 +2074,13 @@
         <v>43</v>
       </c>
       <c r="C37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D37" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E37" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F37">
         <v>4</v>
@@ -2101,7 +2089,7 @@
         <v>4</v>
       </c>
       <c r="H37" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2112,13 +2100,13 @@
         <v>44</v>
       </c>
       <c r="C38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D38" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E38" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F38">
         <v>4</v>
@@ -2127,7 +2115,7 @@
         <v>4</v>
       </c>
       <c r="H38" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2138,13 +2126,13 @@
         <v>45</v>
       </c>
       <c r="C39" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D39" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E39" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -2153,7 +2141,7 @@
         <v>4</v>
       </c>
       <c r="H39" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -2161,16 +2149,16 @@
         <v>46</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C40" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D40" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E40" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F40">
         <v>4</v>
@@ -2179,7 +2167,7 @@
         <v>4</v>
       </c>
       <c r="H40" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2190,13 +2178,13 @@
         <v>47</v>
       </c>
       <c r="C41" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D41" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E41" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F41">
         <v>4</v>
@@ -2205,7 +2193,7 @@
         <v>4</v>
       </c>
       <c r="H41" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -2213,16 +2201,16 @@
         <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D42" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E42" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F42">
         <v>4</v>
@@ -2231,7 +2219,7 @@
         <v>4</v>
       </c>
       <c r="H42" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2242,13 +2230,13 @@
         <v>49</v>
       </c>
       <c r="C43" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D43" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E43" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F43">
         <v>4</v>
@@ -2257,7 +2245,7 @@
         <v>4</v>
       </c>
       <c r="H43" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2268,13 +2256,13 @@
         <v>50</v>
       </c>
       <c r="C44" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D44" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E44" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F44">
         <v>4</v>
@@ -2283,7 +2271,7 @@
         <v>4</v>
       </c>
       <c r="H44" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2294,13 +2282,13 @@
         <v>51</v>
       </c>
       <c r="C45" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D45" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E45" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F45">
         <v>4</v>
@@ -2309,7 +2297,7 @@
         <v>4</v>
       </c>
       <c r="H45" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2317,16 +2305,16 @@
         <v>52</v>
       </c>
       <c r="B46" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C46" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D46" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E46" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F46">
         <v>4</v>
@@ -2335,7 +2323,7 @@
         <v>4</v>
       </c>
       <c r="H46" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -2343,16 +2331,16 @@
         <v>53</v>
       </c>
       <c r="B47" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C47" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D47" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E47" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F47">
         <v>3</v>
@@ -2361,7 +2349,7 @@
         <v>3</v>
       </c>
       <c r="H47" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2372,13 +2360,13 @@
         <v>54</v>
       </c>
       <c r="C48" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D48" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E48" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F48">
         <v>3</v>
@@ -2387,7 +2375,7 @@
         <v>3</v>
       </c>
       <c r="H48" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -2398,13 +2386,13 @@
         <v>55</v>
       </c>
       <c r="C49" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D49" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E49" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F49">
         <v>3</v>
@@ -2413,7 +2401,7 @@
         <v>3</v>
       </c>
       <c r="H49" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -2424,13 +2412,13 @@
         <v>56</v>
       </c>
       <c r="C50" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D50" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E50" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F50">
         <v>3</v>
@@ -2439,7 +2427,7 @@
         <v>3</v>
       </c>
       <c r="H50" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2450,13 +2438,13 @@
         <v>57</v>
       </c>
       <c r="C51" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D51" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E51" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F51">
         <v>3</v>
@@ -2465,7 +2453,7 @@
         <v>3</v>
       </c>
       <c r="H51" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2476,13 +2464,13 @@
         <v>58</v>
       </c>
       <c r="C52" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D52" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E52" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F52">
         <v>3</v>
@@ -2491,7 +2479,7 @@
         <v>3</v>
       </c>
       <c r="H52" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -2502,13 +2490,13 @@
         <v>59</v>
       </c>
       <c r="C53" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D53" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E53" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F53">
         <v>3</v>
@@ -2517,7 +2505,7 @@
         <v>3</v>
       </c>
       <c r="H53" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2528,13 +2516,13 @@
         <v>60</v>
       </c>
       <c r="C54" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D54" t="s">
-        <v>182</v>
+        <v>149</v>
       </c>
       <c r="E54" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F54">
         <v>3</v>
@@ -2543,7 +2531,7 @@
         <v>3</v>
       </c>
       <c r="H54" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2554,13 +2542,13 @@
         <v>61</v>
       </c>
       <c r="C55" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D55" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="E55" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F55">
         <v>3</v>
@@ -2569,7 +2557,7 @@
         <v>3</v>
       </c>
       <c r="H55" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2577,16 +2565,16 @@
         <v>62</v>
       </c>
       <c r="B56" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="C56" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D56" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="E56" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F56">
         <v>3</v>
@@ -2595,7 +2583,7 @@
         <v>3</v>
       </c>
       <c r="H56" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -2603,16 +2591,16 @@
         <v>63</v>
       </c>
       <c r="B57" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="C57" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D57" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="E57" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F57">
         <v>3</v>
@@ -2621,7 +2609,7 @@
         <v>3</v>
       </c>
       <c r="H57" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2629,16 +2617,16 @@
         <v>64</v>
       </c>
       <c r="B58" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="C58" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D58" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="E58" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F58">
         <v>3</v>
@@ -2647,7 +2635,7 @@
         <v>3</v>
       </c>
       <c r="H58" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2655,16 +2643,16 @@
         <v>65</v>
       </c>
       <c r="B59" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="C59" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D59" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="E59" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F59">
         <v>3</v>
@@ -2673,7 +2661,7 @@
         <v>3</v>
       </c>
       <c r="H59" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2684,13 +2672,13 @@
         <v>66</v>
       </c>
       <c r="C60" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D60" t="s">
-        <v>163</v>
+        <v>183</v>
       </c>
       <c r="E60" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F60">
         <v>3</v>
@@ -2699,7 +2687,7 @@
         <v>3</v>
       </c>
       <c r="H60" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -2710,13 +2698,13 @@
         <v>67</v>
       </c>
       <c r="C61" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D61" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E61" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F61">
         <v>3</v>
@@ -2725,7 +2713,7 @@
         <v>3</v>
       </c>
       <c r="H61" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -2736,13 +2724,13 @@
         <v>68</v>
       </c>
       <c r="C62" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D62" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E62" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F62">
         <v>3</v>
@@ -2751,7 +2739,7 @@
         <v>3</v>
       </c>
       <c r="H62" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -2762,13 +2750,13 @@
         <v>69</v>
       </c>
       <c r="C63" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D63" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E63" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F63">
         <v>3</v>
@@ -2777,7 +2765,7 @@
         <v>3</v>
       </c>
       <c r="H63" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -2788,13 +2776,13 @@
         <v>70</v>
       </c>
       <c r="C64" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D64" t="s">
-        <v>189</v>
+        <v>170</v>
       </c>
       <c r="E64" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F64">
         <v>3</v>
@@ -2803,7 +2791,7 @@
         <v>3</v>
       </c>
       <c r="H64" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -2814,13 +2802,13 @@
         <v>71</v>
       </c>
       <c r="C65" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D65" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E65" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F65">
         <v>3</v>
@@ -2829,33 +2817,7 @@
         <v>3</v>
       </c>
       <c r="H65" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8">
-      <c r="A66" t="s">
-        <v>72</v>
-      </c>
-      <c r="B66" t="s">
-        <v>72</v>
-      </c>
-      <c r="C66" t="s">
-        <v>148</v>
-      </c>
-      <c r="D66" t="s">
-        <v>178</v>
-      </c>
-      <c r="E66" t="s">
-        <v>191</v>
-      </c>
-      <c r="F66">
-        <v>3</v>
-      </c>
-      <c r="G66">
-        <v>3</v>
-      </c>
-      <c r="H66" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>